<commit_message>
Calculadora Cafetería Móvil: «ticket» → «precio medio por taza» / «tique» (autotest 1.122 verde)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/calculadora-escandallo-presupuesto-cafe-eventos.xlsx
+++ b/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/calculadora-escandallo-presupuesto-cafe-eventos.xlsx
@@ -2352,7 +2352,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Ticket medio sin IVA de tu carta (€)</t>
+          <t>Precio medio por taza sin IVA de tu carta (€)</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -2374,7 +2374,7 @@
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>El coste con envase es el de la bebida servida en vaso de un solo uso; en loza solo cuenta el coste de producto. Los vasos de papel con forro de PE o PLA ("compostables") son plástico a efectos de la Ley 7/2022: se cobran aparte en el ticket. El food cost del plan financiero es otra cosa: la media de la mezcla con la merma.</t>
+          <t>El coste con envase es el de la bebida servida en vaso de un solo uso; en loza solo cuenta el coste de producto. Los vasos de papel con forro de PE o PLA ("compostables") son plástico a efectos de la Ley 7/2022: se cobran aparte en el tique. El food cost del plan financiero es otra cosa: la media de la mezcla con la merma.</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Loza: sin coste de vaso ni tapa. Vaso de un solo uso: suma el envase y, en el ticket, el precio aparte del vaso de plástico (Ley 7/2022, art. 55). El compostable con forro de PE o PLA también es plástico.</t>
+          <t>Loza: sin coste de vaso ni tapa. Vaso de un solo uso: suma el envase y, en el tique, el precio aparte del vaso de plástico (Ley 7/2022, art. 55). El compostable con forro de PE o PLA también es plástico.</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Feria: ticket medio por taza que cobrarás (sin IVA)</t>
+          <t>Feria: precio medio por taza que cobrarás (sin IVA)</t>
         </is>
       </c>
       <c r="B22" s="13" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Research §4: ≈ 3,00 € sin IVA por taza. Mira el ticket medio de tu carta en la hoja «Escandallo». Solo cuenta si el cliente es Feria.</t>
+          <t>Research §4: ≈ 3,00 € sin IVA por taza. Mira el precio medio por taza de tu carta en la hoja «Escandallo». Solo cuenta si el cliente es Feria.</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Coste ÷ (1 − margen − canon) ÷ invitados, redondeado a los 0,50 € de arriba. Es el precio de las empresas («+ IVA»). En Feria es el ticket mínimo por taza que cubre coste, canon y margen: compáralo con el tuyo.</t>
+          <t>Coste ÷ (1 − margen − canon) ÷ invitados, redondeado a los 0,50 € de arriba. Es el precio de las empresas («+ IVA»). En Feria es el precio mínimo por taza que cubre coste, canon y margen: compáralo con el tuyo.</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Venta prevista (tazas × ticket, sin IVA)</t>
+          <t>Venta prevista (tazas × precio medio, sin IVA)</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -5200,7 +5200,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Feria: ticket medio por taza que cobrarás (sin IVA)</t>
+          <t>Feria: precio medio por taza que cobrarás (sin IVA)</t>
         </is>
       </c>
       <c r="B22" s="20" t="n">
@@ -6307,7 +6307,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Venta prevista (tazas × ticket, sin IVA)</t>
+          <t>Venta prevista (tazas × precio medio, sin IVA)</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Feria: 250 tazas en una jornada de 10 horas, vaso de un solo uso (con su precio aparte en el ticket), generador y canon del 15 % del organizador. El «precio por invitado» es el ticket mínimo por taza; con el ticket de 3,00 € la jornada deja unos 128 € antes de costes fijos, y por debajo de 181 tazas pierdes.</t>
+          <t>Feria: 250 tazas en una jornada de 10 horas, vaso de un solo uso (con su precio aparte en el tique), generador y canon del 15 % del organizador. El «precio por invitado» es el precio mínimo por taza; con un precio medio de 3,00 € la jornada deja unos 128 € antes de costes fijos, y por debajo de 181 tazas pierdes.</t>
         </is>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
     <row r="20" ht="75" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>La bebida para consumir en el acto o para llevar va al 10 % de IVA (Ley 37/1992, art. 91). Los extras con precio propio (personalización de máquina o stand, vasos con logo, talleres) van al 21 %. En loza no hay vaso de plástico; el vaso de papel con forro de PE o PLA («compostable») es plástico a efectos de la Ley 7/2022 (arts. 2 y 55) y se cobra aparte en el ticket. Pajitas y agitadores de plástico, prohibidos. En ferias y festivales, el organizador puede imponer su sistema de vaso reutilizable (RD 1055/2022, art. 7).</t>
+          <t>La bebida para consumir en el acto o para llevar va al 10 % de IVA (Ley 37/1992, art. 91). Los extras con precio propio (personalización de máquina o stand, vasos con logo, talleres) van al 21 %. En loza no hay vaso de plástico; el vaso de papel con forro de PE o PLA («compostable») es plástico a efectos de la Ley 7/2022 (arts. 2 y 55) y se cobra aparte en el tique. Pajitas y agitadores de plástico, prohibidos. En ferias y festivales, el organizador puede imponer su sistema de vaso reutilizable (RD 1055/2022, art. 7).</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>La venta directa en mercados y ferias depende de la autorización municipal y del canon del organizador. La hoja calcula la venta (tazas × ticket), el canon (porcentaje más cuota fija), el resultado de la jornada y las tazas que necesitas para cubrir los costes. El «precio por invitado» de esa columna es el ticket mínimo por taza que cubre coste, canon y margen.</t>
+          <t>La venta directa en mercados y ferias depende de la autorización municipal y del canon del organizador. La hoja calcula la venta (tazas × precio medio), el canon (porcentaje más cuota fija), el resultado de la jornada y las tazas que necesitas para cubrir los costes. El «precio por invitado» de esa columna es el precio mínimo por taza que cubre coste, canon y margen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Calculadora Cafetería Móvil: arreglos de la revisión (M3 sin referencias internas, m22 1.840 h, m23 rótulo del tramo 4)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/calculadora-escandallo-presupuesto-cafe-eventos.xlsx
+++ b/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/calculadora-escandallo-presupuesto-cafe-eventos.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Research §3.b: un doble de especialidad lleva 16-18 g. Mueve los gramos de la fila del café de todas las bebidas.</t>
+          <t>Estimación del kit: un doble de especialidad lleva 16-18 g. Mueve los gramos de la fila del café de todas las bebidas.</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>Research §3.b: 18-28 €/kg, caso 22 €/kg [estimado]; 10 % de merma por purga y calibrado.</t>
+          <t>Estimación del kit: 18-28 €/kg en hostelería, se toma 22 €/kg; 10 % de merma por purga y calibrado.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="O15" s="16" t="inlineStr">
         <is>
-          <t>Research §3.b: ≈ 1,05 €/l [estimado].</t>
+          <t>Estimación del kit: ≈ 1,05 €/l.</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="O17" s="16" t="inlineStr">
         <is>
-          <t>Research §3.b: ≈ 2,50 €/l [estimado].</t>
+          <t>Estimación del kit: ≈ 2,50 €/l.</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>Research §3.b: vaso, tapa, servilleta y removedor ≈ 0,13 € por bebida [cálculo].</t>
+          <t>Estimación del kit: vaso, tapa, servilleta y removedor suman ≈ 0,13 € por bebida.</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Horario</t>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Mañana +25 %, boda de noche −10 % (research §1). Ajusta las bebidas por invitado. En Feria no se usa.</t>
+          <t>Mañana +25 %, boda de noche −10 % (estimación del kit con ratios de EE. UU.). Ajusta las bebidas por invitado. En Feria no se usa.</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Horas por persona fuera del servicio (carga, viaje, montaje y limpieza)</t>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Estimación del kit: un servicio de dos horas es una jornada de siete a nueve (research §1). Pon las reales.</t>
+          <t>Estimación del kit: un servicio de dos horas es una jornada de siete a nueve. Pon las reales.</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Estimación del kit: del titular (14,2 €/h) y del camarero fijo discontinuo (11,0 €/h) con 14 pagas y 1.780 horas. Copia tu convenio.</t>
+          <t>Estimación del kit: del titular (13,7 €/h) y del camarero fijo discontinuo (10,7 €/h) con 14 pagas y 1.840 horas (40 h × 46 semanas, como el plan). Copia tu convenio.</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Research §4: ≈ 3,00 € sin IVA por taza. Mira el precio medio por taza de tu carta en la hoja «Escandallo». Solo cuenta si el cliente es Feria.</t>
+          <t>Estimación del kit: ≈ 3,00 € sin IVA por taza. Mira el precio medio por taza de tu carta en la hoja «Escandallo». Solo cuenta si el cliente es Feria.</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>SPEC D11: un enchufe de 16 A a 230 V da unos 3,7 kW (3,68). Los molinos, la nevera y la iluminación van aparte: déjales margen.</t>
+          <t>Un enchufe de 16 A a 230 V da unos 3,7 kW (3,68). Los molinos, la nevera y la iluminación van aparte: déjales margen.</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Importe que retienes si cancela ese día</t>
+          <t>Importe que retienes si cancela ese día (en el último tramo, antes de descontar los costes que te ahorras)</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -3649,7 +3649,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>REGLAS DE ESCALADO (fuente única: «datos_escalado»; misma tabla que las Instrucciones del plan y el Word)</t>
+          <t>REGLAS DE ESCALADO (la misma tabla que las Instrucciones del plan financiero y el plan de negocio)</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Research: 50-60 bebidas por hora con un barista en dos grupos; con dos baristas, 100-120 (ratios de EE. UU.). Se toma 55.</t>
+          <t>Ratios de EE. UU. (grindkit y beanandbrewtech): 50-60 bebidas por hora con un barista en dos grupos; con dos baristas, 100-120. Se toma 55.</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Research: con dos baristas en una cafetera se llega a 100-120 bebidas por hora; una segunda estación entra por encima de eso.</t>
+          <t>Ratios de EE. UU.: con dos baristas en una cafetera se llega a 100-120 bebidas por hora; una segunda estación entra por encima de eso.</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Research §4: molinos de espresso bajo demanda más uno de descafeinado o filtro.</t>
+          <t>Estimación del kit: un molino de espresso por estación más uno de descafeinado o filtro.</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Research: 100-200 g por evento. Se toma 150 g.</t>
+          <t>Estimación del kit: 100-200 g por evento. Se toma 150 g.</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Del caso: loza para 150 en una boda de 120 invitados (research §4).</t>
+          <t>Del caso: loza para 150 en una boda de 120 invitados (plan financiero).</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Un enchufe de 16 A a 230 V da unos 3,7 kW (3,68 kW): SPEC D11.</t>
+          <t>Un enchufe de 16 A a 230 V da unos 3,7 kW (3,68 kW).</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Margen de arranque: una cafetera de 3,5 kW pide un generador inverter de 5 kVA (research §0).</t>
+          <t>Margen de arranque: una cafetera de 3,5 kW pide un generador inverter de 5 kVA (fichas de distribuidor).</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>Rango del research: 1,0</t>
+          <t>Rango de referencia: 1,0</t>
         </is>
       </c>
       <c r="D107" s="25" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="C108" s="16" t="inlineStr">
         <is>
-          <t>Rango del research: 1,3-1,5</t>
+          <t>Rango de referencia: 1,3-1,5</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C109" s="16" t="inlineStr">
         <is>
-          <t>Rango del research: 1,5-1,8</t>
+          <t>Rango de referencia: 1,5-1,8</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="C110" s="16" t="inlineStr">
         <is>
-          <t>Rango del research: 2,0-2,5</t>
+          <t>Rango de referencia: 2,0-2,5</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="C111" s="16" t="inlineStr">
         <is>
-          <t>Rango del research: mezcla del caso</t>
+          <t>Rango de referencia: mezcla del caso</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="30" customHeight="1">
+    <row r="129" ht="45" customHeight="1">
       <c r="A129" s="4" t="inlineStr">
         <is>
           <t>Canon del organizador (% de la venta)</t>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Solo ferias, mercados y festivales (research §3.a: porcentaje de la venta o cuota fija). El canon fijo se escribe aparte.</t>
+          <t>Solo ferias, mercados y festivales (porcentaje de la venta o cuota fija, según el organizador). El canon fijo se escribe aparte.</t>
         </is>
       </c>
     </row>
@@ -6186,7 +6186,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Importe que retienes si cancela ese día</t>
+          <t>Importe que retienes si cancela ese día (en el último tramo, antes de descontar los costes que te ahorras)</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -6628,7 +6628,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Fuentes: research del producto (octubre 2026); Ley 37/1992 del IVA, art. 91; Ley 7/2022, arts. 2, 55 y 56; RD 1055/2022, art. 7; TRLGDCU, arts. 85, 87 y 103.</t>
+          <t>Fuentes: investigación de AI Chef Pro (octubre 2026); Ley 37/1992 del IVA, art. 91; Ley 7/2022, arts. 2, 55 y 56; RD 1055/2022, art. 7; TRLGDCU, arts. 85, 87 y 103.</t>
         </is>
       </c>
     </row>

</xml_diff>